<commit_message>
fix: excel tagihan seed
</commit_message>
<xml_diff>
--- a/Data_Tagihan.xlsx
+++ b/Data_Tagihan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muham\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1BD82B-CE52-460F-9E8D-5F1049D4AF2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350C160B-8AF7-4D05-956B-17BEBF8883B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{13AFA879-8ABF-49A1-915B-E29C5DB46594}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{13AFA879-8ABF-49A1-915B-E29C5DB46594}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="273">
   <si>
     <t xml:space="preserve">Rezky Nanda Hendrata </t>
   </si>
@@ -104,15 +102,9 @@
     <t xml:space="preserve">AA18-1 </t>
   </si>
   <si>
-    <t>AA18-14</t>
-  </si>
-  <si>
     <t>AA5-17</t>
   </si>
   <si>
-    <t>AA5-16</t>
-  </si>
-  <si>
     <t>AA18-6</t>
   </si>
   <si>
@@ -125,18 +117,9 @@
     <t>AA20-1</t>
   </si>
   <si>
-    <t>AA23-6</t>
-  </si>
-  <si>
-    <t>AA14-30</t>
-  </si>
-  <si>
     <t>AA26-11</t>
   </si>
   <si>
-    <t>AA5-14</t>
-  </si>
-  <si>
     <t>AA27-11</t>
   </si>
   <si>
@@ -173,9 +156,6 @@
     <t xml:space="preserve">KETERANGAN </t>
   </si>
   <si>
-    <t xml:space="preserve">AA5-16 </t>
-  </si>
-  <si>
     <t xml:space="preserve">Ramona </t>
   </si>
   <si>
@@ -185,18 +165,12 @@
     <t xml:space="preserve">Rezky Nanda </t>
   </si>
   <si>
-    <t>AA5-18</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yulianto </t>
   </si>
   <si>
     <t>Reni Sinaga</t>
   </si>
   <si>
-    <t>AA27-8</t>
-  </si>
-  <si>
     <t>Fathul Huda</t>
   </si>
   <si>
@@ -413,9 +387,6 @@
     <t>JenniDp</t>
   </si>
   <si>
-    <t>AA15-6</t>
-  </si>
-  <si>
     <t>Patricia2</t>
   </si>
   <si>
@@ -569,9 +540,6 @@
     <t>Ratih3</t>
   </si>
   <si>
-    <t>AA15-9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Emillia Rosiani </t>
   </si>
   <si>
@@ -815,9 +783,6 @@
     <t>Rumsinah2</t>
   </si>
   <si>
-    <t>AA14-32</t>
-  </si>
-  <si>
     <t>Evi4</t>
   </si>
   <si>
@@ -839,9 +804,6 @@
     <t>Raafita3</t>
   </si>
   <si>
-    <t>AA18-5</t>
-  </si>
-  <si>
     <t>Irma5</t>
   </si>
   <si>
@@ -885,6 +847,12 @@
   </si>
   <si>
     <t>Anom6</t>
+  </si>
+  <si>
+    <t>AA18-12</t>
+  </si>
+  <si>
+    <t>AA23-7</t>
   </si>
 </sst>
 </file>
@@ -1041,9 +1009,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1081,7 +1049,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1187,7 +1155,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1329,7 +1297,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1350,22 +1318,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="9" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1379,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E2" s="17">
         <v>177600000</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1405,7 +1373,7 @@
         <v>226200000</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1425,7 +1393,7 @@
         <v>226200000</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1433,7 +1401,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>3</v>
@@ -1445,7 +1413,7 @@
         <v>29200000</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1453,7 +1421,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>3</v>
@@ -1465,7 +1433,7 @@
         <v>200000000</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1473,7 +1441,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>4</v>
@@ -1485,7 +1453,7 @@
         <v>306200000</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1493,7 +1461,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>24</v>
+        <v>180</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>5</v>
@@ -1505,7 +1473,7 @@
         <v>373000000</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1513,7 +1481,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>6</v>
@@ -1525,7 +1493,7 @@
         <v>26200000</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1533,7 +1501,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>6</v>
@@ -1545,7 +1513,7 @@
         <v>200000000</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1553,7 +1521,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>7</v>
@@ -1565,7 +1533,7 @@
         <v>226200000</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1573,7 +1541,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>8</v>
@@ -1585,7 +1553,7 @@
         <v>226200000</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1593,10 +1561,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D13" s="2">
         <v>45986</v>
@@ -1605,7 +1573,7 @@
         <v>55000000</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1613,10 +1581,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D14" s="2">
         <v>46008</v>
@@ -1625,7 +1593,7 @@
         <v>200000000</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1633,7 +1601,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>29</v>
+        <v>272</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>9</v>
@@ -1645,7 +1613,7 @@
         <v>5000000</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1653,7 +1621,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>29</v>
+        <v>272</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>9</v>
@@ -1665,13 +1633,13 @@
         <v>5000000</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="6" t="s">
-        <v>29</v>
+        <v>272</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>9</v>
@@ -1683,7 +1651,7 @@
         <v>5000000</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1691,7 +1659,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>30</v>
+        <v>138</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>10</v>
@@ -1703,7 +1671,7 @@
         <v>324200000</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1711,7 +1679,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>11</v>
@@ -1723,7 +1691,7 @@
         <v>190600000</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1731,7 +1699,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>12</v>
@@ -1743,7 +1711,7 @@
         <v>306200000</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1751,7 +1719,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>13</v>
@@ -1763,7 +1731,7 @@
         <v>226200000</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1771,7 +1739,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>14</v>
@@ -1783,7 +1751,7 @@
         <v>181400000</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1791,7 +1759,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>15</v>
@@ -1803,7 +1771,7 @@
         <v>328200000</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1811,7 +1779,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>16</v>
@@ -1823,7 +1791,7 @@
         <v>250000000</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1831,7 +1799,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>16</v>
@@ -1843,7 +1811,7 @@
         <v>136800000</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1851,7 +1819,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>17</v>
@@ -1863,7 +1831,7 @@
         <v>152200000</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1871,7 +1839,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>17</v>
@@ -1883,7 +1851,7 @@
         <v>24000000</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1891,7 +1859,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>18</v>
@@ -1903,7 +1871,7 @@
         <v>173160000</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1911,7 +1879,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>45</v>
+        <v>180</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>5</v>
@@ -1923,7 +1891,7 @@
         <v>33333333</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1931,10 +1899,10 @@
         <v>28</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D30" s="2">
         <v>46047</v>
@@ -1943,7 +1911,7 @@
         <v>32500000</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1963,7 +1931,7 @@
         <v>28900000</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1971,7 +1939,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>6</v>
@@ -1983,7 +1951,7 @@
         <v>28900000</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1991,7 +1959,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>3</v>
@@ -2003,7 +1971,7 @@
         <v>28650000</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2011,7 +1979,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>8</v>
@@ -2023,7 +1991,7 @@
         <v>28900000</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2034,7 +2002,7 @@
         <v>19</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D35" s="2">
         <v>46038</v>
@@ -2043,7 +2011,7 @@
         <v>22200000</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2051,7 +2019,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>17</v>
@@ -2063,7 +2031,7 @@
         <v>22650000</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2071,10 +2039,10 @@
         <v>35</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D37" s="2">
         <v>46059</v>
@@ -2083,7 +2051,7 @@
         <v>38900000</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2091,7 +2059,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C38" s="13" t="s">
         <v>8</v>
@@ -2103,7 +2071,7 @@
         <v>28900000</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2111,10 +2079,10 @@
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D39" s="2">
         <v>46059</v>
@@ -2123,7 +2091,7 @@
         <v>38900000</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2131,7 +2099,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C40" s="13" t="s">
         <v>13</v>
@@ -2143,7 +2111,7 @@
         <v>28900000</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2151,10 +2119,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D41" s="2">
         <v>46043</v>
@@ -2163,7 +2131,7 @@
         <v>7000000</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2171,7 +2139,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C42" s="13" t="s">
         <v>17</v>
@@ -2183,7 +2151,7 @@
         <v>22650000</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2191,7 +2159,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>15</v>
@@ -2203,7 +2171,7 @@
         <v>41650000</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2211,7 +2179,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>11</v>
@@ -2223,7 +2191,7 @@
         <v>24450000</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2231,10 +2199,10 @@
         <v>43</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D45" s="2">
         <v>46073</v>
@@ -2243,7 +2211,7 @@
         <v>7000000</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2251,7 +2219,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>14</v>
@@ -2263,7 +2231,7 @@
         <v>23300000</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2274,7 +2242,7 @@
         <v>19</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="D47" s="2">
         <v>46074</v>
@@ -2283,7 +2251,7 @@
         <v>22200000</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2291,7 +2259,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>30</v>
+        <v>138</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>10</v>
@@ -2303,7 +2271,7 @@
         <v>41150000</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2311,10 +2279,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D49" s="2">
         <v>46078</v>
@@ -2323,7 +2291,7 @@
         <v>32500000</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2343,7 +2311,7 @@
         <v>28900000</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2351,7 +2319,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>18</v>
@@ -2363,7 +2331,7 @@
         <v>22270000</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2371,7 +2339,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>3</v>
@@ -2383,7 +2351,7 @@
         <v>28650000</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2391,7 +2359,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>24</v>
+        <v>180</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>5</v>
@@ -2403,7 +2371,7 @@
         <v>33333333</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2411,10 +2379,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D54" s="2">
         <v>46083</v>
@@ -2423,7 +2391,7 @@
         <v>188200000</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2431,7 +2399,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C55" s="11" t="s">
         <v>8</v>
@@ -2443,7 +2411,7 @@
         <v>28900000</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2451,10 +2419,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D56" s="2">
         <v>46116</v>
@@ -2463,7 +2431,7 @@
         <v>38900000</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2471,10 +2439,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D57" s="2">
         <v>46088</v>
@@ -2483,7 +2451,7 @@
         <v>152200000</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2491,10 +2459,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D58" s="2">
         <v>46088</v>
@@ -2503,7 +2471,7 @@
         <v>152200000</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2511,10 +2479,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D59" s="2">
         <v>46088</v>
@@ -2523,7 +2491,7 @@
         <v>163800000</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2531,7 +2499,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C60" s="11" t="s">
         <v>13</v>
@@ -2543,7 +2511,7 @@
         <v>28900000</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2551,10 +2519,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D61" s="2">
         <v>46089</v>
@@ -2563,7 +2531,7 @@
         <v>273400000</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2571,7 +2539,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>15</v>
@@ -2583,7 +2551,7 @@
         <v>41650000</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2591,19 +2559,19 @@
         <v>61</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="E63" s="18">
         <v>7000000</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2614,16 +2582,16 @@
         <v>19</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="E64" s="18">
         <v>22200000</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2631,19 +2599,19 @@
         <v>63</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C65" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E65" s="18">
         <v>23300000</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2657,13 +2625,13 @@
         <v>1</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E66" s="18">
         <v>28900000</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2671,19 +2639,19 @@
         <v>65</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E67" s="18">
         <v>32500000</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2691,19 +2659,19 @@
         <v>66</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C68" s="11" t="s">
         <v>6</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E68" s="18">
         <v>28900000</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2711,19 +2679,19 @@
         <v>67</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C69" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E69" s="18">
         <v>28650000</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2731,19 +2699,19 @@
         <v>68</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="C70" s="11" t="s">
         <v>18</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="E70" s="18">
         <v>22270000</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2751,19 +2719,19 @@
         <v>69</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>24</v>
+        <v>180</v>
       </c>
       <c r="C71" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E71" s="18">
         <v>33333333</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2771,19 +2739,19 @@
         <v>70</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E72" s="18">
         <v>24500000</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2791,19 +2759,19 @@
         <v>71</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C73" s="11" t="s">
         <v>17</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E73" s="18">
         <v>22650000</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2811,19 +2779,19 @@
         <v>72</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C74" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="E74" s="18">
         <v>41150000</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2831,10 +2799,10 @@
         <v>73</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D75" s="2">
         <v>46026</v>
@@ -2843,7 +2811,7 @@
         <v>24150000</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2851,10 +2819,10 @@
         <v>74</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D76" s="2">
         <v>46085</v>
@@ -2863,7 +2831,7 @@
         <v>19650000</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2871,10 +2839,10 @@
         <v>75</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D77" s="2">
         <v>46146</v>
@@ -2883,7 +2851,7 @@
         <v>21100000</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2891,7 +2859,7 @@
         <v>76</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C78" s="11" t="s">
         <v>7</v>
@@ -2903,7 +2871,7 @@
         <v>28900000</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2911,7 +2879,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C79" s="11" t="s">
         <v>8</v>
@@ -2923,7 +2891,7 @@
         <v>28900000</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2931,7 +2899,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>12</v>
@@ -2943,7 +2911,7 @@
         <v>38900000</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2951,7 +2919,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C81" s="11" t="s">
         <v>16</v>
@@ -2963,7 +2931,7 @@
         <v>21766667</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2971,7 +2939,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>17</v>
@@ -2983,7 +2951,7 @@
         <v>22650000</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -2991,10 +2959,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D83" s="2">
         <v>46207</v>
@@ -3003,7 +2971,7 @@
         <v>19650000</v>
       </c>
       <c r="F83" s="6" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -3011,7 +2979,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>15</v>
@@ -3023,7 +2991,7 @@
         <v>41650000</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -3031,7 +2999,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>13</v>
@@ -3043,7 +3011,7 @@
         <v>28900000</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -3051,19 +3019,19 @@
         <v>84</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="E86" s="18">
         <v>211200000</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3071,19 +3039,19 @@
         <v>85</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>7</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="E87" s="18">
         <v>28900000</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3091,19 +3059,19 @@
         <v>86</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="E88" s="18">
         <v>38900000</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -3111,19 +3079,19 @@
         <v>87</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E89" s="18">
         <v>7000000</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3134,16 +3102,16 @@
         <v>19</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="E90" s="18">
         <v>22200000</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3151,19 +3119,19 @@
         <v>89</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E91" s="18">
         <v>34800000</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -3171,19 +3139,19 @@
         <v>90</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C92" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E92" s="18">
         <v>23300000</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3191,19 +3159,19 @@
         <v>91</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>177</v>
+        <v>218</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="E93" s="18">
         <v>324200000</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -3211,19 +3179,19 @@
         <v>92</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="E94" s="18">
         <v>248200000</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -3231,19 +3199,19 @@
         <v>93</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E95" s="18">
         <v>32500000</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -3257,13 +3225,13 @@
         <v>1</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E96" s="18">
         <v>28900000</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3271,19 +3239,19 @@
         <v>95</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C97" s="11" t="s">
         <v>6</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E97" s="18">
         <v>28900000</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3291,19 +3259,19 @@
         <v>96</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>22</v>
+        <v>271</v>
       </c>
       <c r="C98" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="E98" s="18">
         <v>28650000</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3311,19 +3279,19 @@
         <v>97</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C99" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="E99" s="18">
         <v>33333333</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3331,10 +3299,10 @@
         <v>98</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D100" s="2">
         <v>46086</v>
@@ -3343,7 +3311,7 @@
         <v>100000000</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3351,7 +3319,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C101" s="11" t="s">
         <v>10</v>
@@ -3363,7 +3331,7 @@
         <v>41150000</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3371,7 +3339,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>8</v>
@@ -3383,7 +3351,7 @@
         <v>28900000</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -3391,10 +3359,10 @@
         <v>101</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D103" s="2">
         <v>46178</v>
@@ -3403,7 +3371,7 @@
         <v>38900000</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -3411,7 +3379,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C104" s="11" t="s">
         <v>17</v>
@@ -3423,7 +3391,7 @@
         <v>22650000</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -3431,7 +3399,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C105" s="11" t="s">
         <v>16</v>
@@ -3443,7 +3411,7 @@
         <v>21766667</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3451,7 +3419,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C106" s="11" t="s">
         <v>16</v>
@@ -3463,7 +3431,7 @@
         <v>21766667</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -3471,7 +3439,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C107" s="11" t="s">
         <v>16</v>
@@ -3483,7 +3451,7 @@
         <v>21766667</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -3491,19 +3459,19 @@
         <v>106</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C108" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E108" s="18">
         <v>24500000</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3511,10 +3479,10 @@
         <v>107</v>
       </c>
       <c r="B109" s="7" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C109" s="11" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D109" s="2">
         <v>46300</v>
@@ -3523,7 +3491,7 @@
         <v>19650000</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3531,7 +3499,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="C110" s="11" t="s">
         <v>15</v>
@@ -3543,7 +3511,7 @@
         <v>41650000</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3551,7 +3519,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C111" s="11" t="s">
         <v>7</v>
@@ -3563,7 +3531,7 @@
         <v>28900000</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -3571,7 +3539,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C112" s="11" t="s">
         <v>13</v>
@@ -3583,7 +3551,7 @@
         <v>28900000</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -3594,16 +3562,16 @@
         <v>19</v>
       </c>
       <c r="C113" s="11" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E113" s="18">
         <v>22200000</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3611,19 +3579,19 @@
         <v>112</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C114" s="11" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E114" s="18">
         <v>34800000</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -3631,19 +3599,19 @@
         <v>113</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C115" s="11" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="E115" s="18">
         <v>118100000</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -3651,19 +3619,19 @@
         <v>114</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="C116" s="11" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="E116" s="18">
         <v>250000000</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -3671,19 +3639,19 @@
         <v>115</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C117" s="11" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="E117" s="18">
         <v>250000000</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -3691,19 +3659,19 @@
         <v>116</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="C118" s="11" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="E118" s="18">
         <v>100000000</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -3711,19 +3679,19 @@
         <v>117</v>
       </c>
       <c r="B119" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C119" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="D119" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="C119" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="E119" s="18">
         <v>250000000</v>
       </c>
       <c r="F119" s="6" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -3731,19 +3699,19 @@
         <v>118</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="E120" s="18">
         <v>82300000</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -3751,19 +3719,19 @@
         <v>119</v>
       </c>
       <c r="B121" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C121" s="11" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="E121" s="18">
         <v>100000000</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -3771,19 +3739,19 @@
         <v>120</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="C122" s="11" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="E122" s="18">
         <v>16400000</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -3791,19 +3759,19 @@
         <v>121</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="E123" s="18">
         <v>224200000</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -3811,19 +3779,19 @@
         <v>122</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C124" s="11" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="E124" s="18">
         <v>100000000</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -3831,19 +3799,19 @@
         <v>123</v>
       </c>
       <c r="B125" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C125" s="11" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="E125" s="18">
         <v>24450000</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -3851,19 +3819,19 @@
         <v>124</v>
       </c>
       <c r="B126" s="7" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="C126" s="11" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="E126" s="18">
         <v>100000000</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -3871,19 +3839,19 @@
         <v>125</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C127" s="11" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E127" s="18">
         <v>32500000</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -3891,19 +3859,19 @@
         <v>126</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C128" s="11" t="s">
         <v>6</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E128" s="18">
         <v>28900000</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -3911,19 +3879,19 @@
         <v>127</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C129" s="11" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E129" s="18">
         <v>100000000</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -3931,19 +3899,19 @@
         <v>128</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C130" s="11" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E130" s="18">
         <v>50000000</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -3951,19 +3919,19 @@
         <v>129</v>
       </c>
       <c r="B131" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C131" s="11" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E131" s="18">
         <v>38900000</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -3971,19 +3939,19 @@
         <v>130</v>
       </c>
       <c r="B132" s="7" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C132" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="E132" s="18">
         <v>33333333</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -3997,13 +3965,13 @@
         <v>1</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="E133" s="18">
         <v>28900000</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -4011,19 +3979,19 @@
         <v>132</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="E134" s="18">
         <v>7000000</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -4031,19 +3999,19 @@
         <v>133</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="C135" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="E135" s="18">
         <v>23300000</v>
       </c>
       <c r="F135" s="6" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -4051,10 +4019,10 @@
         <v>134</v>
       </c>
       <c r="B136" s="7" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D136" s="2">
         <v>46028</v>
@@ -4063,7 +4031,7 @@
         <v>19650000</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -4071,7 +4039,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="7" t="s">
-        <v>259</v>
+        <v>138</v>
       </c>
       <c r="C137" s="11" t="s">
         <v>10</v>
@@ -4083,7 +4051,7 @@
         <v>41150000</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -4091,10 +4059,10 @@
         <v>136</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D138" s="2">
         <v>46028</v>
@@ -4103,7 +4071,7 @@
         <v>34800000</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -4111,10 +4079,10 @@
         <v>137</v>
       </c>
       <c r="B139" s="7" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="D139" s="2">
         <v>46028</v>
@@ -4123,7 +4091,7 @@
         <v>150000000</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
@@ -4131,10 +4099,10 @@
         <v>138</v>
       </c>
       <c r="B140" s="7" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D140" s="2">
         <v>46028</v>
@@ -4143,7 +4111,7 @@
         <v>24150000</v>
       </c>
       <c r="F140" s="6" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
@@ -4151,10 +4119,10 @@
         <v>139</v>
       </c>
       <c r="B141" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="C141" s="11" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D141" s="2">
         <v>46059</v>
@@ -4163,7 +4131,7 @@
         <v>21100000</v>
       </c>
       <c r="F141" s="6" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
@@ -4171,7 +4139,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="7" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>3</v>
@@ -4183,7 +4151,7 @@
         <v>28650000</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
@@ -4191,10 +4159,10 @@
         <v>141</v>
       </c>
       <c r="B143" s="7" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="C143" s="11" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="D143" s="2">
         <v>46179</v>
@@ -4203,7 +4171,7 @@
         <v>280000000</v>
       </c>
       <c r="F143" s="6" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
@@ -4211,7 +4179,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>8</v>
@@ -4223,7 +4191,7 @@
         <v>28900000</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
@@ -4231,10 +4199,10 @@
         <v>143</v>
       </c>
       <c r="B145" s="7" t="s">
-        <v>32</v>
+        <v>188</v>
       </c>
       <c r="C145" s="11" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D145" s="2">
         <v>46148</v>
@@ -4243,7 +4211,7 @@
         <v>38900000</v>
       </c>
       <c r="F145" s="6" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
@@ -4251,10 +4219,10 @@
         <v>144</v>
       </c>
       <c r="B146" s="7" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="C146" s="11" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="D146" s="2">
         <v>46179</v>
@@ -4263,7 +4231,7 @@
         <v>176200000</v>
       </c>
       <c r="F146" s="6" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -4271,10 +4239,10 @@
         <v>145</v>
       </c>
       <c r="B147" s="7" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C147" s="11" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D147" s="2">
         <v>46209</v>
@@ -4283,7 +4251,7 @@
         <v>19650000</v>
       </c>
       <c r="F147" s="6" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -4291,7 +4259,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C148" s="11" t="s">
         <v>13</v>
@@ -4303,7 +4271,7 @@
         <v>28900000</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
@@ -4311,7 +4279,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C149" s="11" t="s">
         <v>17</v>
@@ -4323,7 +4291,7 @@
         <v>22650000</v>
       </c>
       <c r="F149" s="6" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
@@ -4331,10 +4299,10 @@
         <v>148</v>
       </c>
       <c r="B150" s="7" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C150" s="11" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D150" s="2">
         <v>46240</v>
@@ -4343,7 +4311,7 @@
         <v>19650000</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -4351,10 +4319,10 @@
         <v>149</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C151" s="11" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D151" s="2">
         <v>46271</v>
@@ -4363,7 +4331,7 @@
         <v>35300000</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
@@ -4371,7 +4339,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C152" s="11" t="s">
         <v>16</v>
@@ -4383,7 +4351,7 @@
         <v>21766667</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -4391,7 +4359,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C153" s="11" t="s">
         <v>16</v>
@@ -4403,7 +4371,7 @@
         <v>21766667</v>
       </c>
       <c r="F153" s="6" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: excel tagihan seed 2
</commit_message>
<xml_diff>
--- a/Data_Tagihan.xlsx
+++ b/Data_Tagihan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muham\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\aku\code\kerjaan\2026\kavling-web\kavling-backend-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350C160B-8AF7-4D05-956B-17BEBF8883B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{151CA9F4-5480-42B5-A734-1E42FF15A9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{13AFA879-8ABF-49A1-915B-E29C5DB46594}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="272">
   <si>
     <t xml:space="preserve">Rezky Nanda Hendrata </t>
   </si>
@@ -109,9 +109,6 @@
   </si>
   <si>
     <t>AA20-6</t>
-  </si>
-  <si>
-    <t>AA19-9</t>
   </si>
   <si>
     <t>AA20-1</t>
@@ -1318,22 +1315,22 @@
   <sheetData>
     <row r="1" spans="1:6" s="9" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1347,13 +1344,13 @@
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E2" s="17">
         <v>177600000</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1373,7 +1370,7 @@
         <v>226200000</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1393,7 +1390,7 @@
         <v>226200000</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1401,7 +1398,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>3</v>
@@ -1413,7 +1410,7 @@
         <v>29200000</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1421,7 +1418,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>3</v>
@@ -1433,7 +1430,7 @@
         <v>200000000</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1453,7 +1450,7 @@
         <v>306200000</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1461,7 +1458,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>5</v>
@@ -1473,7 +1470,7 @@
         <v>373000000</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1493,7 +1490,7 @@
         <v>26200000</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1513,7 +1510,7 @@
         <v>200000000</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1533,7 +1530,7 @@
         <v>226200000</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1541,7 +1538,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>8</v>
@@ -1553,7 +1550,7 @@
         <v>226200000</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1561,10 +1558,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2">
         <v>45986</v>
@@ -1573,7 +1570,7 @@
         <v>55000000</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1581,10 +1578,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2">
         <v>46008</v>
@@ -1593,7 +1590,7 @@
         <v>200000000</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1601,7 +1598,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>9</v>
@@ -1613,7 +1610,7 @@
         <v>5000000</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1621,7 +1618,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>9</v>
@@ -1633,13 +1630,13 @@
         <v>5000000</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>9</v>
@@ -1651,7 +1648,7 @@
         <v>5000000</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1659,7 +1656,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>10</v>
@@ -1671,7 +1668,7 @@
         <v>324200000</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1679,7 +1676,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>11</v>
@@ -1691,7 +1688,7 @@
         <v>190600000</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1699,7 +1696,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>12</v>
@@ -1711,7 +1708,7 @@
         <v>306200000</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1719,7 +1716,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>13</v>
@@ -1731,7 +1728,7 @@
         <v>226200000</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1739,7 +1736,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>14</v>
@@ -1751,7 +1748,7 @@
         <v>181400000</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1759,7 +1756,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>15</v>
@@ -1771,7 +1768,7 @@
         <v>328200000</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1779,7 +1776,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>16</v>
@@ -1791,7 +1788,7 @@
         <v>250000000</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1799,7 +1796,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>16</v>
@@ -1811,7 +1808,7 @@
         <v>136800000</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1819,7 +1816,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>17</v>
@@ -1831,7 +1828,7 @@
         <v>152200000</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1839,7 +1836,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>17</v>
@@ -1851,7 +1848,7 @@
         <v>24000000</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1859,7 +1856,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>18</v>
@@ -1871,7 +1868,7 @@
         <v>173160000</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1879,7 +1876,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>5</v>
@@ -1891,7 +1888,7 @@
         <v>33333333</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1899,10 +1896,10 @@
         <v>28</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D30" s="2">
         <v>46047</v>
@@ -1911,7 +1908,7 @@
         <v>32500000</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1931,7 +1928,7 @@
         <v>28900000</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1951,7 +1948,7 @@
         <v>28900000</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1959,7 +1956,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>3</v>
@@ -1971,7 +1968,7 @@
         <v>28650000</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1979,7 +1976,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>8</v>
@@ -1991,7 +1988,7 @@
         <v>28900000</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2002,7 +1999,7 @@
         <v>19</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" s="2">
         <v>46038</v>
@@ -2011,7 +2008,7 @@
         <v>22200000</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2019,7 +2016,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>17</v>
@@ -2031,7 +2028,7 @@
         <v>22650000</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2042,7 +2039,7 @@
         <v>22</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D37" s="2">
         <v>46059</v>
@@ -2051,7 +2048,7 @@
         <v>38900000</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2059,7 +2056,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C38" s="13" t="s">
         <v>8</v>
@@ -2071,7 +2068,7 @@
         <v>28900000</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2079,10 +2076,10 @@
         <v>37</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D39" s="2">
         <v>46059</v>
@@ -2091,7 +2088,7 @@
         <v>38900000</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2099,7 +2096,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C40" s="13" t="s">
         <v>13</v>
@@ -2111,7 +2108,7 @@
         <v>28900000</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2119,10 +2116,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D41" s="2">
         <v>46043</v>
@@ -2131,7 +2128,7 @@
         <v>7000000</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2139,7 +2136,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C42" s="13" t="s">
         <v>17</v>
@@ -2151,7 +2148,7 @@
         <v>22650000</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2159,7 +2156,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>15</v>
@@ -2171,7 +2168,7 @@
         <v>41650000</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2179,7 +2176,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>11</v>
@@ -2191,7 +2188,7 @@
         <v>24450000</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2199,10 +2196,10 @@
         <v>43</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D45" s="2">
         <v>46073</v>
@@ -2211,7 +2208,7 @@
         <v>7000000</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2219,7 +2216,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>14</v>
@@ -2231,7 +2228,7 @@
         <v>23300000</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2242,7 +2239,7 @@
         <v>19</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D47" s="2">
         <v>46074</v>
@@ -2251,7 +2248,7 @@
         <v>22200000</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2259,7 +2256,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>10</v>
@@ -2271,7 +2268,7 @@
         <v>41150000</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2279,10 +2276,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D49" s="2">
         <v>46078</v>
@@ -2291,7 +2288,7 @@
         <v>32500000</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2311,7 +2308,7 @@
         <v>28900000</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2319,7 +2316,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>18</v>
@@ -2331,7 +2328,7 @@
         <v>22270000</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2339,7 +2336,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>3</v>
@@ -2351,7 +2348,7 @@
         <v>28650000</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2359,7 +2356,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>5</v>
@@ -2371,7 +2368,7 @@
         <v>33333333</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2379,10 +2376,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C54" s="11" t="s">
         <v>99</v>
-      </c>
-      <c r="C54" s="11" t="s">
-        <v>100</v>
       </c>
       <c r="D54" s="2">
         <v>46083</v>
@@ -2391,7 +2388,7 @@
         <v>188200000</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2399,7 +2396,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C55" s="11" t="s">
         <v>8</v>
@@ -2411,7 +2408,7 @@
         <v>28900000</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2419,10 +2416,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D56" s="2">
         <v>46116</v>
@@ -2431,7 +2428,7 @@
         <v>38900000</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2439,10 +2436,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C57" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="C57" s="11" t="s">
-        <v>105</v>
       </c>
       <c r="D57" s="2">
         <v>46088</v>
@@ -2451,7 +2448,7 @@
         <v>152200000</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2459,10 +2456,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="C58" s="11" t="s">
-        <v>108</v>
       </c>
       <c r="D58" s="2">
         <v>46088</v>
@@ -2471,7 +2468,7 @@
         <v>152200000</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2479,10 +2476,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C59" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D59" s="2">
         <v>46088</v>
@@ -2491,7 +2488,7 @@
         <v>163800000</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2499,7 +2496,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C60" s="11" t="s">
         <v>13</v>
@@ -2511,7 +2508,7 @@
         <v>28900000</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2519,10 +2516,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>114</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="D61" s="2">
         <v>46089</v>
@@ -2531,7 +2528,7 @@
         <v>273400000</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2539,7 +2536,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>15</v>
@@ -2551,7 +2548,7 @@
         <v>41650000</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2559,19 +2556,19 @@
         <v>61</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E63" s="18">
         <v>7000000</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2582,16 +2579,16 @@
         <v>19</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E64" s="18">
         <v>22200000</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2599,19 +2596,19 @@
         <v>63</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C65" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E65" s="18">
         <v>23300000</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2625,13 +2622,13 @@
         <v>1</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E66" s="18">
         <v>28900000</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2639,19 +2636,19 @@
         <v>65</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E67" s="18">
         <v>32500000</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2665,13 +2662,13 @@
         <v>6</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E68" s="18">
         <v>28900000</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2679,19 +2676,19 @@
         <v>67</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C69" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E69" s="18">
         <v>28650000</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2699,19 +2696,19 @@
         <v>68</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C70" s="11" t="s">
         <v>18</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E70" s="18">
         <v>22270000</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2719,19 +2716,19 @@
         <v>69</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C71" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E71" s="18">
         <v>33333333</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2739,19 +2736,19 @@
         <v>70</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E72" s="18">
         <v>24500000</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2759,19 +2756,19 @@
         <v>71</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C73" s="11" t="s">
         <v>17</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E73" s="18">
         <v>22650000</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2779,19 +2776,19 @@
         <v>72</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C74" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E74" s="18">
         <v>41150000</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2799,10 +2796,10 @@
         <v>73</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D75" s="2">
         <v>46026</v>
@@ -2811,7 +2808,7 @@
         <v>24150000</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2819,10 +2816,10 @@
         <v>74</v>
       </c>
       <c r="B76" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C76" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>108</v>
       </c>
       <c r="D76" s="2">
         <v>46085</v>
@@ -2831,7 +2828,7 @@
         <v>19650000</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2839,10 +2836,10 @@
         <v>75</v>
       </c>
       <c r="B77" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C77" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="C77" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D77" s="2">
         <v>46146</v>
@@ -2851,7 +2848,7 @@
         <v>21100000</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2871,7 +2868,7 @@
         <v>28900000</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2879,7 +2876,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C79" s="11" t="s">
         <v>8</v>
@@ -2891,7 +2888,7 @@
         <v>28900000</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2899,7 +2896,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>12</v>
@@ -2911,7 +2908,7 @@
         <v>38900000</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2919,7 +2916,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C81" s="11" t="s">
         <v>16</v>
@@ -2931,7 +2928,7 @@
         <v>21766667</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2939,7 +2936,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>17</v>
@@ -2951,7 +2948,7 @@
         <v>22650000</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -2959,10 +2956,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C83" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="C83" s="11" t="s">
-        <v>105</v>
       </c>
       <c r="D83" s="2">
         <v>46207</v>
@@ -2971,7 +2968,7 @@
         <v>19650000</v>
       </c>
       <c r="F83" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -2979,7 +2976,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>15</v>
@@ -2991,7 +2988,7 @@
         <v>41650000</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -2999,7 +2996,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>13</v>
@@ -3011,7 +3008,7 @@
         <v>28900000</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -3019,19 +3016,19 @@
         <v>84</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E86" s="18">
         <v>211200000</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3045,13 +3042,13 @@
         <v>7</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E87" s="18">
         <v>28900000</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3062,16 +3059,16 @@
         <v>22</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E88" s="18">
         <v>38900000</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -3079,19 +3076,19 @@
         <v>87</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E89" s="18">
         <v>7000000</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3102,16 +3099,16 @@
         <v>19</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E90" s="18">
         <v>22200000</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3119,19 +3116,19 @@
         <v>89</v>
       </c>
       <c r="B91" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C91" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="C91" s="11" t="s">
-        <v>115</v>
-      </c>
       <c r="D91" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E91" s="18">
         <v>34800000</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -3139,19 +3136,19 @@
         <v>90</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C92" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E92" s="18">
         <v>23300000</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3159,19 +3156,19 @@
         <v>91</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C93" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>169</v>
       </c>
       <c r="E93" s="18">
         <v>324200000</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -3179,19 +3176,19 @@
         <v>92</v>
       </c>
       <c r="B94" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C94" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="C94" s="11" t="s">
-        <v>172</v>
-      </c>
       <c r="D94" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E94" s="18">
         <v>248200000</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -3199,19 +3196,19 @@
         <v>93</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E95" s="18">
         <v>32500000</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -3225,13 +3222,13 @@
         <v>1</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E96" s="18">
         <v>28900000</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3245,13 +3242,13 @@
         <v>6</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E97" s="18">
         <v>28900000</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3259,19 +3256,19 @@
         <v>96</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C98" s="11" t="s">
         <v>3</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E98" s="18">
         <v>28650000</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3279,19 +3276,19 @@
         <v>97</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C99" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E99" s="18">
         <v>33333333</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3299,10 +3296,10 @@
         <v>98</v>
       </c>
       <c r="B100" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C100" s="11" t="s">
         <v>183</v>
-      </c>
-      <c r="C100" s="11" t="s">
-        <v>184</v>
       </c>
       <c r="D100" s="2">
         <v>46086</v>
@@ -3311,7 +3308,7 @@
         <v>100000000</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3319,7 +3316,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C101" s="11" t="s">
         <v>10</v>
@@ -3331,7 +3328,7 @@
         <v>41150000</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3339,7 +3336,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>8</v>
@@ -3351,7 +3348,7 @@
         <v>28900000</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -3359,10 +3356,10 @@
         <v>101</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D103" s="2">
         <v>46178</v>
@@ -3371,7 +3368,7 @@
         <v>38900000</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -3379,7 +3376,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C104" s="11" t="s">
         <v>17</v>
@@ -3391,7 +3388,7 @@
         <v>22650000</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -3399,7 +3396,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C105" s="11" t="s">
         <v>16</v>
@@ -3411,7 +3408,7 @@
         <v>21766667</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3419,7 +3416,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C106" s="11" t="s">
         <v>16</v>
@@ -3431,7 +3428,7 @@
         <v>21766667</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -3439,7 +3436,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C107" s="11" t="s">
         <v>16</v>
@@ -3451,7 +3448,7 @@
         <v>21766667</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -3459,19 +3456,19 @@
         <v>106</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C108" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E108" s="18">
         <v>24500000</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3479,10 +3476,10 @@
         <v>107</v>
       </c>
       <c r="B109" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C109" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="C109" s="11" t="s">
-        <v>108</v>
       </c>
       <c r="D109" s="2">
         <v>46300</v>
@@ -3491,7 +3488,7 @@
         <v>19650000</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3499,7 +3496,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C110" s="11" t="s">
         <v>15</v>
@@ -3511,7 +3508,7 @@
         <v>41650000</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3531,7 +3528,7 @@
         <v>28900000</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -3539,7 +3536,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C112" s="11" t="s">
         <v>13</v>
@@ -3551,7 +3548,7 @@
         <v>28900000</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -3562,16 +3559,16 @@
         <v>19</v>
       </c>
       <c r="C113" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E113" s="18">
         <v>22200000</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3579,19 +3576,19 @@
         <v>112</v>
       </c>
       <c r="B114" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C114" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="C114" s="11" t="s">
-        <v>115</v>
-      </c>
       <c r="D114" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E114" s="18">
         <v>34800000</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -3599,19 +3596,19 @@
         <v>113</v>
       </c>
       <c r="B115" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C115" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C115" s="11" t="s">
+      <c r="D115" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>205</v>
       </c>
       <c r="E115" s="18">
         <v>118100000</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -3619,19 +3616,19 @@
         <v>114</v>
       </c>
       <c r="B116" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="C116" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="C116" s="11" t="s">
-        <v>208</v>
-      </c>
       <c r="D116" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E116" s="18">
         <v>250000000</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -3639,19 +3636,19 @@
         <v>115</v>
       </c>
       <c r="B117" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C117" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="C117" s="11" t="s">
-        <v>211</v>
-      </c>
       <c r="D117" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E117" s="18">
         <v>250000000</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -3659,19 +3656,19 @@
         <v>116</v>
       </c>
       <c r="B118" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C118" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="C118" s="11" t="s">
+      <c r="D118" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>215</v>
       </c>
       <c r="E118" s="18">
         <v>100000000</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -3679,19 +3676,19 @@
         <v>117</v>
       </c>
       <c r="B119" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="C119" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="C119" s="11" t="s">
-        <v>208</v>
-      </c>
       <c r="D119" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E119" s="18">
         <v>250000000</v>
       </c>
       <c r="F119" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -3699,19 +3696,19 @@
         <v>118</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E120" s="18">
         <v>82300000</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -3719,19 +3716,19 @@
         <v>119</v>
       </c>
       <c r="B121" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C121" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="C121" s="11" t="s">
-        <v>184</v>
-      </c>
       <c r="D121" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E121" s="18">
         <v>100000000</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -3739,19 +3736,19 @@
         <v>120</v>
       </c>
       <c r="B122" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C122" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="D122" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="C122" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="E122" s="18">
         <v>16400000</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -3759,19 +3756,19 @@
         <v>121</v>
       </c>
       <c r="B123" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C123" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="C123" s="11" t="s">
-        <v>226</v>
-      </c>
       <c r="D123" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E123" s="18">
         <v>224200000</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -3779,19 +3776,19 @@
         <v>122</v>
       </c>
       <c r="B124" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C124" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="C124" s="11" t="s">
-        <v>184</v>
-      </c>
       <c r="D124" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E124" s="18">
         <v>100000000</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -3799,19 +3796,19 @@
         <v>123</v>
       </c>
       <c r="B125" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C125" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E125" s="18">
         <v>24450000</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -3819,19 +3816,19 @@
         <v>124</v>
       </c>
       <c r="B126" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C126" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="C126" s="11" t="s">
-        <v>226</v>
-      </c>
       <c r="D126" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E126" s="18">
         <v>100000000</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -3839,19 +3836,19 @@
         <v>125</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C127" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E127" s="18">
         <v>32500000</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -3865,13 +3862,13 @@
         <v>6</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E128" s="18">
         <v>28900000</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -3879,19 +3876,19 @@
         <v>127</v>
       </c>
       <c r="B129" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C129" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="C129" s="11" t="s">
-        <v>184</v>
-      </c>
       <c r="D129" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E129" s="18">
         <v>100000000</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -3899,19 +3896,19 @@
         <v>128</v>
       </c>
       <c r="B130" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C130" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="C130" s="11" t="s">
-        <v>184</v>
-      </c>
       <c r="D130" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E130" s="18">
         <v>50000000</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -3922,16 +3919,16 @@
         <v>22</v>
       </c>
       <c r="C131" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E131" s="18">
         <v>38900000</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -3939,19 +3936,19 @@
         <v>130</v>
       </c>
       <c r="B132" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C132" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E132" s="18">
         <v>33333333</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -3965,13 +3962,13 @@
         <v>1</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E133" s="18">
         <v>28900000</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -3979,19 +3976,19 @@
         <v>132</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E134" s="18">
         <v>7000000</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -3999,19 +3996,19 @@
         <v>133</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C135" s="11" t="s">
         <v>14</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E135" s="18">
         <v>23300000</v>
       </c>
       <c r="F135" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -4019,10 +4016,10 @@
         <v>134</v>
       </c>
       <c r="B136" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C136" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="C136" s="11" t="s">
-        <v>105</v>
       </c>
       <c r="D136" s="2">
         <v>46028</v>
@@ -4031,7 +4028,7 @@
         <v>19650000</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -4039,7 +4036,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C137" s="11" t="s">
         <v>10</v>
@@ -4051,7 +4048,7 @@
         <v>41150000</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -4059,10 +4056,10 @@
         <v>136</v>
       </c>
       <c r="B138" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C138" s="11" t="s">
         <v>114</v>
-      </c>
-      <c r="C138" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="D138" s="2">
         <v>46028</v>
@@ -4071,7 +4068,7 @@
         <v>34800000</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -4079,10 +4076,10 @@
         <v>137</v>
       </c>
       <c r="B139" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C139" s="11" t="s">
         <v>251</v>
-      </c>
-      <c r="C139" s="11" t="s">
-        <v>252</v>
       </c>
       <c r="D139" s="2">
         <v>46028</v>
@@ -4091,7 +4088,7 @@
         <v>150000000</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
@@ -4099,10 +4096,10 @@
         <v>138</v>
       </c>
       <c r="B140" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D140" s="2">
         <v>46028</v>
@@ -4111,7 +4108,7 @@
         <v>24150000</v>
       </c>
       <c r="F140" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
@@ -4119,10 +4116,10 @@
         <v>139</v>
       </c>
       <c r="B141" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C141" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="C141" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="D141" s="2">
         <v>46059</v>
@@ -4131,7 +4128,7 @@
         <v>21100000</v>
       </c>
       <c r="F141" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
@@ -4139,7 +4136,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>3</v>
@@ -4151,7 +4148,7 @@
         <v>28650000</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
@@ -4159,10 +4156,10 @@
         <v>141</v>
       </c>
       <c r="B143" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C143" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D143" s="2">
         <v>46179</v>
@@ -4171,7 +4168,7 @@
         <v>280000000</v>
       </c>
       <c r="F143" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
@@ -4179,7 +4176,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>8</v>
@@ -4191,7 +4188,7 @@
         <v>28900000</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
@@ -4199,10 +4196,10 @@
         <v>143</v>
       </c>
       <c r="B145" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C145" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D145" s="2">
         <v>46148</v>
@@ -4211,7 +4208,7 @@
         <v>38900000</v>
       </c>
       <c r="F145" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
@@ -4219,10 +4216,10 @@
         <v>144</v>
       </c>
       <c r="B146" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="C146" s="11" t="s">
         <v>261</v>
-      </c>
-      <c r="C146" s="11" t="s">
-        <v>262</v>
       </c>
       <c r="D146" s="2">
         <v>46179</v>
@@ -4231,7 +4228,7 @@
         <v>176200000</v>
       </c>
       <c r="F146" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -4239,10 +4236,10 @@
         <v>145</v>
       </c>
       <c r="B147" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C147" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="C147" s="11" t="s">
-        <v>108</v>
       </c>
       <c r="D147" s="2">
         <v>46209</v>
@@ -4251,7 +4248,7 @@
         <v>19650000</v>
       </c>
       <c r="F147" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -4259,7 +4256,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C148" s="11" t="s">
         <v>13</v>
@@ -4271,7 +4268,7 @@
         <v>28900000</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
@@ -4279,7 +4276,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C149" s="11" t="s">
         <v>17</v>
@@ -4291,7 +4288,7 @@
         <v>22650000</v>
       </c>
       <c r="F149" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
@@ -4299,10 +4296,10 @@
         <v>148</v>
       </c>
       <c r="B150" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C150" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="C150" s="11" t="s">
-        <v>105</v>
       </c>
       <c r="D150" s="2">
         <v>46240</v>
@@ -4311,7 +4308,7 @@
         <v>19650000</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -4319,10 +4316,10 @@
         <v>149</v>
       </c>
       <c r="B151" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C151" s="11" t="s">
         <v>210</v>
-      </c>
-      <c r="C151" s="11" t="s">
-        <v>211</v>
       </c>
       <c r="D151" s="2">
         <v>46271</v>
@@ -4331,7 +4328,7 @@
         <v>35300000</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
@@ -4339,7 +4336,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C152" s="11" t="s">
         <v>16</v>
@@ -4351,7 +4348,7 @@
         <v>21766667</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -4359,7 +4356,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C153" s="11" t="s">
         <v>16</v>
@@ -4371,7 +4368,7 @@
         <v>21766667</v>
       </c>
       <c r="F153" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>